<commit_message>
Add LAR and Kredit yang Diberikan
</commit_message>
<xml_diff>
--- a/data/summarized fitur Kualitas Aset - KBMI 4.xlsx
+++ b/data/summarized fitur Kualitas Aset - KBMI 4.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M89"/>
+  <dimension ref="A1:N89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,6 +496,11 @@
       <c r="M1" s="1" t="inlineStr">
         <is>
           <t>laba_per_kredit_restruk</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>total_npl_dan_restruk_npl_per_kredit_yang_diberikan</t>
         </is>
       </c>
     </row>
@@ -539,6 +544,7 @@
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -580,6 +586,7 @@
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -621,6 +628,7 @@
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -662,6 +670,7 @@
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -711,6 +720,9 @@
       <c r="M6" t="n">
         <v>2.980267361365033</v>
       </c>
+      <c r="N6" t="n">
+        <v>0.01339041781402988</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -760,6 +772,9 @@
       <c r="M7" t="n">
         <v>0.4418057366323974</v>
       </c>
+      <c r="N7" t="n">
+        <v>0.02377640618634983</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -809,6 +824,9 @@
       <c r="M8" t="n">
         <v>0.4131142856407822</v>
       </c>
+      <c r="N8" t="n">
+        <v>0.02159347271591813</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -858,6 +876,9 @@
       <c r="M9" t="n">
         <v>0.6560680999940406</v>
       </c>
+      <c r="N9" t="n">
+        <v>0.02621469184020214</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -901,6 +922,7 @@
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -944,6 +966,7 @@
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -987,6 +1010,7 @@
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1030,6 +1054,7 @@
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1073,6 +1098,7 @@
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1116,6 +1142,7 @@
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1159,6 +1186,7 @@
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1202,6 +1230,7 @@
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1253,6 +1282,9 @@
       <c r="M18" t="n">
         <v>0.217878344029856</v>
       </c>
+      <c r="N18" t="n">
+        <v>0.01934416360337767</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1304,6 +1336,9 @@
       <c r="M19" t="n">
         <v>0.08392798246644934</v>
       </c>
+      <c r="N19" t="n">
+        <v>0.03470621765868327</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1355,6 +1390,9 @@
       <c r="M20" t="n">
         <v>0.02795410269331179</v>
       </c>
+      <c r="N20" t="n">
+        <v>0.03561493396608476</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1406,6 +1444,9 @@
       <c r="M21" t="n">
         <v>0.05892807491760126</v>
       </c>
+      <c r="N21" t="n">
+        <v>0.03023725365526973</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1457,6 +1498,9 @@
       <c r="M22" t="n">
         <v>0.2695656185149064</v>
       </c>
+      <c r="N22" t="n">
+        <v>0.01793925943396714</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1508,6 +1552,9 @@
       <c r="M23" t="n">
         <v>0.08840545135137037</v>
       </c>
+      <c r="N23" t="n">
+        <v>0.03255082347614852</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1559,6 +1606,9 @@
       <c r="M24" t="n">
         <v>0.01973719425417369</v>
       </c>
+      <c r="N24" t="n">
+        <v>0.04253066783365851</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1610,6 +1660,9 @@
       <c r="M25" t="n">
         <v>0.07958472851295179</v>
       </c>
+      <c r="N25" t="n">
+        <v>0.0293639965945477</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1661,6 +1714,9 @@
       <c r="M26" t="n">
         <v>0.0664499420466062</v>
       </c>
+      <c r="N26" t="n">
+        <v>0.01830717677005279</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1712,6 +1768,9 @@
       <c r="M27" t="n">
         <v>0.03146206619483385</v>
       </c>
+      <c r="N27" t="n">
+        <v>0.03264850170216708</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1763,6 +1822,9 @@
       <c r="M28" t="n">
         <v>0.01790537063076626</v>
       </c>
+      <c r="N28" t="n">
+        <v>0.04121899015693729</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1814,6 +1876,9 @@
       <c r="M29" t="n">
         <v>0.02827750808184887</v>
       </c>
+      <c r="N29" t="n">
+        <v>0.03121617238261164</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1865,6 +1930,9 @@
       <c r="M30" t="n">
         <v>0.1412729336482283</v>
       </c>
+      <c r="N30" t="n">
+        <v>0.02388108352702427</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1916,6 +1984,9 @@
       <c r="M31" t="n">
         <v>0.0716610003634893</v>
       </c>
+      <c r="N31" t="n">
+        <v>0.03148680481284105</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1967,6 +2038,9 @@
       <c r="M32" t="n">
         <v>0.0383625962667371</v>
       </c>
+      <c r="N32" t="n">
+        <v>0.03942461493355728</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2018,6 +2092,9 @@
       <c r="M33" t="n">
         <v>0.05561414194014471</v>
       </c>
+      <c r="N33" t="n">
+        <v>0.03269049545392062</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2069,6 +2146,9 @@
       <c r="M34" t="n">
         <v>0.2671574857220484</v>
       </c>
+      <c r="N34" t="n">
+        <v>0.02361587352437221</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2120,6 +2200,9 @@
       <c r="M35" t="n">
         <v>0.1130417599119455</v>
       </c>
+      <c r="N35" t="n">
+        <v>0.03039272079221194</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2171,6 +2254,9 @@
       <c r="M36" t="n">
         <v>0.06032822026886347</v>
       </c>
+      <c r="N36" t="n">
+        <v>0.03811632397685883</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2222,6 +2308,9 @@
       <c r="M37" t="n">
         <v>0.09547730049400893</v>
       </c>
+      <c r="N37" t="n">
+        <v>0.03290355832417238</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2273,6 +2362,9 @@
       <c r="M38" t="n">
         <v>0.380777515001293</v>
       </c>
+      <c r="N38" t="n">
+        <v>0.0216094839268</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2324,6 +2416,9 @@
       <c r="M39" t="n">
         <v>0.1842286214739941</v>
       </c>
+      <c r="N39" t="n">
+        <v>0.02791752925889613</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2375,6 +2470,9 @@
       <c r="M40" t="n">
         <v>0.08693138170887009</v>
       </c>
+      <c r="N40" t="n">
+        <v>0.03700105986220686</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2426,6 +2524,9 @@
       <c r="M41" t="n">
         <v>0.1567917131837556</v>
       </c>
+      <c r="N41" t="n">
+        <v>0.03082509482676659</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2477,6 +2578,9 @@
       <c r="M42" t="n">
         <v>0.09818516819005334</v>
       </c>
+      <c r="N42" t="n">
+        <v>0.02302558150412579</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -2528,6 +2632,9 @@
       <c r="M43" t="n">
         <v>0.06723192606350017</v>
       </c>
+      <c r="N43" t="n">
+        <v>0.02719963391734079</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2579,6 +2686,9 @@
       <c r="M44" t="n">
         <v>0.03679426179812799</v>
       </c>
+      <c r="N44" t="n">
+        <v>0.03462229671552012</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2630,6 +2740,9 @@
       <c r="M45" t="n">
         <v>0.05657311748227122</v>
       </c>
+      <c r="N45" t="n">
+        <v>0.03153219295044306</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2681,6 +2794,9 @@
       <c r="M46" t="n">
         <v>0.2426513460331705</v>
       </c>
+      <c r="N46" t="n">
+        <v>0.0220730888895202</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2732,6 +2848,9 @@
       <c r="M47" t="n">
         <v>0.1497443938257997</v>
       </c>
+      <c r="N47" t="n">
+        <v>0.02444304503631974</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2783,6 +2902,9 @@
       <c r="M48" t="n">
         <v>0.08366310095738637</v>
       </c>
+      <c r="N48" t="n">
+        <v>0.03157201238912438</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2834,6 +2956,9 @@
       <c r="M49" t="n">
         <v>0.133573364058205</v>
       </c>
+      <c r="N49" t="n">
+        <v>0.03322666745857679</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2885,6 +3010,9 @@
       <c r="M50" t="n">
         <v>0.4075189478196957</v>
       </c>
+      <c r="N50" t="n">
+        <v>0.02161636559739541</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2936,6 +3064,9 @@
       <c r="M51" t="n">
         <v>0.2464978403924094</v>
       </c>
+      <c r="N51" t="n">
+        <v>0.02242955243799912</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2987,6 +3118,9 @@
       <c r="M52" t="n">
         <v>0.1297044979115895</v>
       </c>
+      <c r="N52" t="n">
+        <v>0.03042763951395841</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -3038,6 +3172,9 @@
       <c r="M53" t="n">
         <v>0.2276157674412307</v>
       </c>
+      <c r="N53" t="n">
+        <v>0.0313778279562365</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -3089,6 +3226,9 @@
       <c r="M54" t="n">
         <v>0.6424756048093646</v>
       </c>
+      <c r="N54" t="n">
+        <v>0.01706673775294645</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -3140,6 +3280,9 @@
       <c r="M55" t="n">
         <v>0.3691115309121391</v>
       </c>
+      <c r="N55" t="n">
+        <v>0.01870353056876234</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -3191,6 +3334,9 @@
       <c r="M56" t="n">
         <v>0.2026708596726231</v>
       </c>
+      <c r="N56" t="n">
+        <v>0.02805876375781372</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -3242,6 +3388,9 @@
       <c r="M57" t="n">
         <v>0.3236415579976921</v>
       </c>
+      <c r="N57" t="n">
+        <v>0.02817191414817521</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -3293,6 +3442,9 @@
       <c r="M58" t="n">
         <v>0.1912585933917461</v>
       </c>
+      <c r="N58" t="n">
+        <v>0.01757215339692315</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -3344,6 +3496,9 @@
       <c r="M59" t="n">
         <v>0.1192683365141366</v>
       </c>
+      <c r="N59" t="n">
+        <v>0.01687572238835663</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -3395,6 +3550,9 @@
       <c r="M60" t="n">
         <v>0.05972264445427427</v>
       </c>
+      <c r="N60" t="n">
+        <v>0.02770569313277955</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -3446,6 +3604,9 @@
       <c r="M61" t="n">
         <v>0.09726222299052775</v>
       </c>
+      <c r="N61" t="n">
+        <v>0.0301570231435519</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -3497,6 +3658,9 @@
       <c r="M62" t="n">
         <v>0.4759491403806874</v>
       </c>
+      <c r="N62" t="n">
+        <v>0.01885353811311774</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -3548,6 +3712,9 @@
       <c r="M63" t="n">
         <v>0.2648679660114718</v>
       </c>
+      <c r="N63" t="n">
+        <v>0.01517652489118137</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -3599,6 +3766,9 @@
       <c r="M64" t="n">
         <v>0.1136487750324553</v>
       </c>
+      <c r="N64" t="n">
+        <v>0.0245082933456366</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -3650,6 +3820,9 @@
       <c r="M65" t="n">
         <v>0.2076145977877804</v>
       </c>
+      <c r="N65" t="n">
+        <v>0.03103211912464152</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -3701,6 +3874,9 @@
       <c r="M66" t="n">
         <v>0.7968154337160264</v>
       </c>
+      <c r="N66" t="n">
+        <v>0.02039183350973218</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -3752,6 +3928,9 @@
       <c r="M67" t="n">
         <v>0.431370340115431</v>
       </c>
+      <c r="N67" t="n">
+        <v>0.01353509706436289</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -3803,6 +3982,9 @@
       <c r="M68" t="n">
         <v>0.1937584219735323</v>
       </c>
+      <c r="N68" t="n">
+        <v>0.02268873803711702</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -3854,6 +4036,9 @@
       <c r="M69" t="n">
         <v>0.337112960006638</v>
       </c>
+      <c r="N69" t="n">
+        <v>0.03226783881283395</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -3905,6 +4090,9 @@
       <c r="M70" t="n">
         <v>1.182440029862631</v>
       </c>
+      <c r="N70" t="n">
+        <v>0.0179647707637777</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -3956,6 +4144,9 @@
       <c r="M71" t="n">
         <v>0.653439643418579</v>
       </c>
+      <c r="N71" t="n">
+        <v>0.01013047004089135</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -4007,6 +4198,9 @@
       <c r="M72" t="n">
         <v>0.2762210361233576</v>
       </c>
+      <c r="N72" t="n">
+        <v>0.02138300477601125</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -4058,6 +4252,9 @@
       <c r="M73" t="n">
         <v>0.518527217376455</v>
       </c>
+      <c r="N73" t="n">
+        <v>0.03121340550328582</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -4109,6 +4306,9 @@
       <c r="M74" t="n">
         <v>0.3410618429816317</v>
       </c>
+      <c r="N74" t="n">
+        <v>0.01879070493651482</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -4160,6 +4360,9 @@
       <c r="M75" t="n">
         <v>0.1440770554355168</v>
       </c>
+      <c r="N75" t="n">
+        <v>0.01011755394171578</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -4211,6 +4414,9 @@
       <c r="M76" t="n">
         <v>0.07049771730337492</v>
       </c>
+      <c r="N76" t="n">
+        <v>0.02035093975641137</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -4262,6 +4468,9 @@
       <c r="M77" t="n">
         <v>0.1446760234163869</v>
       </c>
+      <c r="N77" t="n">
+        <v>0.03265448832029902</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -4313,6 +4522,9 @@
       <c r="M78" t="n">
         <v>0.7990374552997899</v>
       </c>
+      <c r="N78" t="n">
+        <v>0.02137745421549851</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -4364,6 +4576,9 @@
       <c r="M79" t="n">
         <v>0.325110929760596</v>
       </c>
+      <c r="N79" t="n">
+        <v>0.01006756373657717</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -4415,6 +4630,9 @@
       <c r="M80" t="n">
         <v>0.1454837416692387</v>
       </c>
+      <c r="N80" t="n">
+        <v>0.01979576743997241</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -4466,6 +4684,9 @@
       <c r="M81" t="n">
         <v>0.3085199276546733</v>
       </c>
+      <c r="N81" t="n">
+        <v>0.03209265511265692</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -4517,6 +4738,9 @@
       <c r="M82" t="n">
         <v>1.244045357935571</v>
       </c>
+      <c r="N82" t="n">
+        <v>0.02054615136636861</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -4568,6 +4792,9 @@
       <c r="M83" t="n">
         <v>0.5331197274206613</v>
       </c>
+      <c r="N83" t="n">
+        <v>0.009677746467296328</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -4619,6 +4846,9 @@
       <c r="M84" t="n">
         <v>0.2250300664095782</v>
       </c>
+      <c r="N84" t="n">
+        <v>0.01973462247290796</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -4670,6 +4900,9 @@
       <c r="M85" t="n">
         <v>0.4672342898344865</v>
       </c>
+      <c r="N85" t="n">
+        <v>0.03040340196862456</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -4721,6 +4954,9 @@
       <c r="M86" t="n">
         <v>1.90041123992335</v>
       </c>
+      <c r="N86" t="n">
+        <v>0.01731792017531394</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -4772,6 +5008,9 @@
       <c r="M87" t="n">
         <v>0.6960460821605844</v>
       </c>
+      <c r="N87" t="n">
+        <v>0.009619649943202266</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -4823,6 +5062,9 @@
       <c r="M88" t="n">
         <v>0.3186333685513322</v>
       </c>
+      <c r="N88" t="n">
+        <v>0.01967725433365103</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -4873,6 +5115,9 @@
       </c>
       <c r="M89" t="n">
         <v>0.6488374673589008</v>
+      </c>
+      <c r="N89" t="n">
+        <v>0.02934733248679442</v>
       </c>
     </row>
   </sheetData>

</xml_diff>